<commit_message>
tercer commit de un caso de pruebas
</commit_message>
<xml_diff>
--- a/alumnos/jose-comba/Casos_de_Prueba.xlsx
+++ b/alumnos/jose-comba/Casos_de_Prueba.xlsx
@@ -1107,7 +1107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1231,7 +1231,17 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1245,12 +1255,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1272,6 +1282,30 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1317,40 +1351,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1712,44 +1718,44 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:15" ht="37.5" customHeight="1" thickBot="1">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="60"/>
+      <c r="C2" s="64"/>
       <c r="D2" s="32"/>
-      <c r="E2" s="59" t="s">
+      <c r="E2" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="60"/>
-      <c r="G2" s="56" t="s">
+      <c r="F2" s="64"/>
+      <c r="G2" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="58"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="61"/>
     </row>
     <row r="3" spans="2:15" ht="16.5" thickBot="1">
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="62"/>
+      <c r="C3" s="66"/>
       <c r="D3" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="61" t="s">
+      <c r="E3" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="62"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="63" t="s">
+      <c r="F3" s="66"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="64"/>
-      <c r="K3" s="53"/>
-      <c r="L3" s="54"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="58"/>
     </row>
     <row r="4" spans="2:15" ht="15.75" thickBot="1">
       <c r="B4" s="23"/>
@@ -1778,27 +1784,27 @@
       <c r="L5" s="22"/>
     </row>
     <row r="6" spans="2:15" ht="33" customHeight="1" thickBot="1">
-      <c r="B6" s="59" t="s">
+      <c r="B6" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="60"/>
+      <c r="C6" s="64"/>
       <c r="D6" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="59" t="s">
+      <c r="E6" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="60"/>
-      <c r="G6" s="65">
+      <c r="F6" s="64"/>
+      <c r="G6" s="69">
         <v>45244</v>
       </c>
-      <c r="H6" s="58"/>
-      <c r="I6" s="63" t="s">
+      <c r="H6" s="61"/>
+      <c r="I6" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="J6" s="64"/>
-      <c r="K6" s="53"/>
-      <c r="L6" s="54"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="57"/>
+      <c r="L6" s="58"/>
     </row>
     <row r="7" spans="2:15" ht="15.75" thickBot="1">
       <c r="B7" s="22"/>
@@ -1817,43 +1823,43 @@
       <c r="B8" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="63" t="s">
+      <c r="C8" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="66"/>
-      <c r="E8" s="64"/>
+      <c r="D8" s="78"/>
+      <c r="E8" s="68"/>
       <c r="F8" s="41"/>
       <c r="G8" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="67" t="s">
+      <c r="H8" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="68"/>
-      <c r="J8" s="68"/>
-      <c r="K8" s="68"/>
-      <c r="L8" s="69"/>
+      <c r="I8" s="80"/>
+      <c r="J8" s="80"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="81"/>
     </row>
     <row r="9" spans="2:15" ht="15.75" thickBot="1">
       <c r="B9" s="44">
         <v>1</v>
       </c>
-      <c r="C9" s="71" t="s">
+      <c r="C9" s="83" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="73"/>
+      <c r="D9" s="84"/>
+      <c r="E9" s="85"/>
       <c r="F9" s="41"/>
       <c r="G9" s="39">
         <v>1</v>
       </c>
-      <c r="H9" s="56" t="s">
+      <c r="H9" s="60" t="s">
         <v>116</v>
       </c>
-      <c r="I9" s="57"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="70"/>
+      <c r="I9" s="62"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="62"/>
+      <c r="L9" s="82"/>
     </row>
     <row r="10" spans="2:15" ht="15.75" customHeight="1" thickBot="1">
       <c r="B10" s="46">
@@ -1866,49 +1872,49 @@
       <c r="G10" s="39">
         <v>2</v>
       </c>
-      <c r="H10" s="56" t="s">
+      <c r="H10" s="60" t="s">
         <v>117</v>
       </c>
-      <c r="I10" s="57"/>
-      <c r="J10" s="57"/>
-      <c r="K10" s="57"/>
-      <c r="L10" s="70"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="62"/>
+      <c r="L10" s="82"/>
     </row>
     <row r="11" spans="2:15" ht="51.75" customHeight="1" thickBot="1">
       <c r="B11" s="45">
         <v>3</v>
       </c>
-      <c r="C11" s="74" t="s">
+      <c r="C11" s="86" t="s">
         <v>118</v>
       </c>
-      <c r="D11" s="75"/>
-      <c r="E11" s="76"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="88"/>
       <c r="F11" s="41"/>
       <c r="G11" s="39">
         <v>3</v>
       </c>
-      <c r="H11" s="53"/>
-      <c r="I11" s="55"/>
-      <c r="J11" s="55"/>
-      <c r="K11" s="55"/>
-      <c r="L11" s="77"/>
+      <c r="H11" s="57"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="59"/>
+      <c r="L11" s="89"/>
     </row>
     <row r="12" spans="2:15" ht="16.5" thickBot="1">
       <c r="B12" s="25">
         <v>4</v>
       </c>
-      <c r="C12" s="53"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="54"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="58"/>
       <c r="F12" s="41"/>
       <c r="G12" s="40">
         <v>4</v>
       </c>
-      <c r="H12" s="78"/>
-      <c r="I12" s="79"/>
-      <c r="J12" s="79"/>
-      <c r="K12" s="79"/>
-      <c r="L12" s="80"/>
+      <c r="H12" s="90"/>
+      <c r="I12" s="91"/>
+      <c r="J12" s="91"/>
+      <c r="K12" s="91"/>
+      <c r="L12" s="92"/>
       <c r="O12" s="6"/>
     </row>
     <row r="13" spans="2:15" ht="15.75">
@@ -1991,519 +1997,511 @@
       <c r="L18" s="27"/>
     </row>
     <row r="19" spans="2:12" ht="15" customHeight="1">
-      <c r="B19" s="81" t="s">
+      <c r="B19" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="83" t="s">
+      <c r="C19" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="84"/>
-      <c r="E19" s="83" t="s">
+      <c r="D19" s="73"/>
+      <c r="E19" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="F19" s="84"/>
-      <c r="G19" s="83" t="s">
+      <c r="F19" s="73"/>
+      <c r="G19" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="87"/>
-      <c r="I19" s="84"/>
-      <c r="J19" s="83" t="s">
+      <c r="H19" s="76"/>
+      <c r="I19" s="73"/>
+      <c r="J19" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="K19" s="87"/>
-      <c r="L19" s="84"/>
+      <c r="K19" s="76"/>
+      <c r="L19" s="73"/>
     </row>
     <row r="20" spans="2:12" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B20" s="82"/>
-      <c r="C20" s="85"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="85"/>
-      <c r="F20" s="86"/>
-      <c r="G20" s="85"/>
-      <c r="H20" s="88"/>
-      <c r="I20" s="86"/>
-      <c r="J20" s="85"/>
-      <c r="K20" s="88"/>
-      <c r="L20" s="86"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="75"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="75"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="75"/>
+      <c r="J20" s="74"/>
+      <c r="K20" s="77"/>
+      <c r="L20" s="75"/>
     </row>
     <row r="21" spans="2:12" ht="93.75" customHeight="1" thickBot="1">
       <c r="B21" s="49">
         <v>1</v>
       </c>
-      <c r="C21" s="53" t="s">
+      <c r="C21" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="D21" s="54"/>
-      <c r="E21" s="56" t="s">
+      <c r="D21" s="58"/>
+      <c r="E21" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="58"/>
-      <c r="G21" s="56" t="s">
+      <c r="F21" s="61"/>
+      <c r="G21" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="H21" s="57"/>
-      <c r="I21" s="58"/>
-      <c r="J21" s="56" t="s">
+      <c r="H21" s="62"/>
+      <c r="I21" s="61"/>
+      <c r="J21" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="K21" s="57"/>
-      <c r="L21" s="58"/>
+      <c r="K21" s="62"/>
+      <c r="L21" s="61"/>
     </row>
     <row r="22" spans="2:12" ht="30" customHeight="1" thickBot="1">
       <c r="B22" s="49">
         <v>2</v>
       </c>
-      <c r="C22" s="56" t="s">
+      <c r="C22" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="58"/>
-      <c r="E22" s="56" t="s">
+      <c r="D22" s="61"/>
+      <c r="E22" s="60" t="s">
         <v>45</v>
       </c>
-      <c r="F22" s="58"/>
-      <c r="G22" s="56" t="s">
+      <c r="F22" s="61"/>
+      <c r="G22" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="H22" s="57"/>
-      <c r="I22" s="58"/>
-      <c r="J22" s="56" t="s">
+      <c r="H22" s="62"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="K22" s="57"/>
-      <c r="L22" s="58"/>
+      <c r="K22" s="62"/>
+      <c r="L22" s="61"/>
     </row>
     <row r="23" spans="2:12" ht="30" customHeight="1" thickBot="1">
       <c r="B23" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="C23" s="56" t="s">
+      <c r="C23" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="58"/>
-      <c r="E23" s="56" t="s">
+      <c r="D23" s="61"/>
+      <c r="E23" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="F23" s="58"/>
-      <c r="G23" s="56" t="s">
+      <c r="F23" s="61"/>
+      <c r="G23" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="H23" s="57"/>
-      <c r="I23" s="58"/>
-      <c r="J23" s="56" t="s">
+      <c r="H23" s="62"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="K23" s="57"/>
-      <c r="L23" s="58"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="61"/>
     </row>
     <row r="24" spans="2:12" ht="68.25" customHeight="1" thickBot="1">
       <c r="B24" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="56" t="s">
+      <c r="C24" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D24" s="58"/>
-      <c r="E24" s="56" t="s">
+      <c r="D24" s="61"/>
+      <c r="E24" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="F24" s="58"/>
-      <c r="G24" s="56" t="s">
+      <c r="F24" s="61"/>
+      <c r="G24" s="60" t="s">
         <v>49</v>
       </c>
-      <c r="H24" s="57"/>
-      <c r="I24" s="58"/>
-      <c r="J24" s="56" t="s">
+      <c r="H24" s="62"/>
+      <c r="I24" s="61"/>
+      <c r="J24" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="K24" s="57"/>
-      <c r="L24" s="58"/>
+      <c r="K24" s="62"/>
+      <c r="L24" s="61"/>
     </row>
     <row r="25" spans="2:12" ht="68.25" customHeight="1" thickBot="1">
       <c r="B25" s="49" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="53" t="s">
+      <c r="C25" s="57" t="s">
         <v>78</v>
       </c>
-      <c r="D25" s="54"/>
-      <c r="E25" s="53" t="s">
+      <c r="D25" s="58"/>
+      <c r="E25" s="57" t="s">
         <v>113</v>
       </c>
-      <c r="F25" s="54"/>
-      <c r="G25" s="53" t="s">
+      <c r="F25" s="58"/>
+      <c r="G25" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="H25" s="55"/>
-      <c r="I25" s="54"/>
-      <c r="J25" s="53" t="s">
+      <c r="H25" s="59"/>
+      <c r="I25" s="58"/>
+      <c r="J25" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="K25" s="55"/>
-      <c r="L25" s="54"/>
+      <c r="K25" s="59"/>
+      <c r="L25" s="58"/>
     </row>
     <row r="26" spans="2:12" ht="49.5" customHeight="1" thickBot="1">
       <c r="B26" s="49" t="s">
         <v>80</v>
       </c>
-      <c r="C26" s="56" t="s">
+      <c r="C26" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D26" s="58"/>
-      <c r="E26" s="56" t="s">
+      <c r="D26" s="61"/>
+      <c r="E26" s="60" t="s">
         <v>114</v>
       </c>
-      <c r="F26" s="58"/>
-      <c r="G26" s="56" t="s">
+      <c r="F26" s="61"/>
+      <c r="G26" s="60" t="s">
         <v>115</v>
       </c>
-      <c r="H26" s="57"/>
-      <c r="I26" s="58"/>
-      <c r="J26" s="56" t="s">
+      <c r="H26" s="62"/>
+      <c r="I26" s="61"/>
+      <c r="J26" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="K26" s="57"/>
-      <c r="L26" s="58"/>
+      <c r="K26" s="62"/>
+      <c r="L26" s="61"/>
     </row>
     <row r="27" spans="2:12" ht="81" customHeight="1" thickBot="1">
       <c r="B27" s="49">
         <v>3</v>
       </c>
-      <c r="C27" s="56" t="s">
+      <c r="C27" s="60" t="s">
         <v>119</v>
       </c>
-      <c r="D27" s="58"/>
-      <c r="E27" s="56" t="s">
+      <c r="D27" s="61"/>
+      <c r="E27" s="60" t="s">
         <v>92</v>
       </c>
-      <c r="F27" s="58"/>
-      <c r="G27" s="56" t="s">
+      <c r="F27" s="61"/>
+      <c r="G27" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="H27" s="57"/>
-      <c r="I27" s="58"/>
-      <c r="J27" s="56" t="s">
+      <c r="H27" s="62"/>
+      <c r="I27" s="61"/>
+      <c r="J27" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="K27" s="57"/>
-      <c r="L27" s="58"/>
+      <c r="K27" s="62"/>
+      <c r="L27" s="61"/>
     </row>
     <row r="28" spans="2:12" ht="46.5" customHeight="1" thickBot="1">
       <c r="B28" s="49" t="s">
         <v>122</v>
       </c>
-      <c r="C28" s="53" t="s">
+      <c r="C28" s="57" t="s">
         <v>120</v>
       </c>
-      <c r="D28" s="54"/>
-      <c r="E28" s="53" t="s">
+      <c r="D28" s="58"/>
+      <c r="E28" s="57" t="s">
         <v>121</v>
       </c>
-      <c r="F28" s="54"/>
-      <c r="G28" s="53" t="s">
+      <c r="F28" s="58"/>
+      <c r="G28" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="H28" s="55"/>
-      <c r="I28" s="54"/>
-      <c r="J28" s="53" t="s">
+      <c r="H28" s="59"/>
+      <c r="I28" s="58"/>
+      <c r="J28" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="K28" s="55"/>
-      <c r="L28" s="54"/>
+      <c r="K28" s="59"/>
+      <c r="L28" s="58"/>
     </row>
     <row r="29" spans="2:12" ht="31.5" customHeight="1" thickBot="1">
       <c r="B29" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="C29" s="53" t="s">
+      <c r="C29" s="57" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="54"/>
-      <c r="E29" s="53" t="s">
+      <c r="D29" s="58"/>
+      <c r="E29" s="57" t="s">
         <v>125</v>
       </c>
-      <c r="F29" s="54"/>
-      <c r="G29" s="53" t="s">
+      <c r="F29" s="58"/>
+      <c r="G29" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="55"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="53" t="s">
+      <c r="H29" s="59"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="K29" s="55"/>
-      <c r="L29" s="54"/>
+      <c r="K29" s="59"/>
+      <c r="L29" s="58"/>
     </row>
     <row r="30" spans="2:12" ht="15.75" customHeight="1" thickBot="1">
       <c r="B30" s="49" t="s">
         <v>103</v>
       </c>
-      <c r="C30" s="53" t="s">
+      <c r="C30" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D30" s="54"/>
-      <c r="E30" s="53" t="s">
+      <c r="D30" s="58"/>
+      <c r="E30" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="F30" s="54"/>
-      <c r="G30" s="53" t="s">
+      <c r="F30" s="58"/>
+      <c r="G30" s="57" t="s">
         <v>41</v>
       </c>
-      <c r="H30" s="55"/>
-      <c r="I30" s="54"/>
-      <c r="J30" s="53" t="s">
+      <c r="H30" s="59"/>
+      <c r="I30" s="58"/>
+      <c r="J30" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="K30" s="55"/>
-      <c r="L30" s="54"/>
+      <c r="K30" s="59"/>
+      <c r="L30" s="58"/>
     </row>
     <row r="31" spans="2:12" ht="32.25" customHeight="1" thickBot="1">
       <c r="B31" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="C31" s="56" t="s">
+      <c r="C31" s="60" t="s">
         <v>126</v>
       </c>
-      <c r="D31" s="58"/>
-      <c r="E31" s="56" t="s">
+      <c r="D31" s="61"/>
+      <c r="E31" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="F31" s="58"/>
-      <c r="G31" s="56" t="s">
+      <c r="F31" s="61"/>
+      <c r="G31" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="H31" s="57"/>
-      <c r="I31" s="58"/>
-      <c r="J31" s="56" t="s">
+      <c r="H31" s="62"/>
+      <c r="I31" s="61"/>
+      <c r="J31" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="K31" s="57"/>
-      <c r="L31" s="58"/>
+      <c r="K31" s="62"/>
+      <c r="L31" s="61"/>
     </row>
     <row r="32" spans="2:12" ht="33" customHeight="1" thickBot="1">
       <c r="B32" s="49" t="s">
         <v>110</v>
       </c>
-      <c r="C32" s="56" t="s">
+      <c r="C32" s="60" t="s">
         <v>127</v>
       </c>
-      <c r="D32" s="58"/>
-      <c r="E32" s="56" t="s">
+      <c r="D32" s="61"/>
+      <c r="E32" s="60" t="s">
         <v>128</v>
       </c>
-      <c r="F32" s="58"/>
-      <c r="G32" s="56" t="s">
+      <c r="F32" s="61"/>
+      <c r="G32" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="H32" s="57"/>
-      <c r="I32" s="58"/>
-      <c r="J32" s="56" t="s">
+      <c r="H32" s="62"/>
+      <c r="I32" s="61"/>
+      <c r="J32" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="K32" s="57"/>
-      <c r="L32" s="58"/>
+      <c r="K32" s="62"/>
+      <c r="L32" s="61"/>
     </row>
     <row r="33" spans="2:12" ht="15.75" thickBot="1">
       <c r="B33" s="49" t="s">
         <v>112</v>
       </c>
-      <c r="C33" s="53" t="s">
+      <c r="C33" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="D33" s="54"/>
-      <c r="E33" s="53" t="s">
+      <c r="D33" s="58"/>
+      <c r="E33" s="57" t="s">
         <v>39</v>
       </c>
-      <c r="F33" s="54"/>
-      <c r="G33" s="53" t="s">
+      <c r="F33" s="58"/>
+      <c r="G33" s="57" t="s">
         <v>129</v>
       </c>
-      <c r="H33" s="55"/>
-      <c r="I33" s="54"/>
-      <c r="J33" s="53" t="s">
+      <c r="H33" s="59"/>
+      <c r="I33" s="58"/>
+      <c r="J33" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="K33" s="55"/>
-      <c r="L33" s="54"/>
+      <c r="K33" s="59"/>
+      <c r="L33" s="58"/>
     </row>
     <row r="34" spans="2:12" ht="15.75" customHeight="1" thickBot="1">
       <c r="B34" s="49"/>
-      <c r="C34" s="53"/>
-      <c r="D34" s="54"/>
-      <c r="E34" s="53"/>
-      <c r="F34" s="54"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="54"/>
-      <c r="J34" s="53"/>
-      <c r="K34" s="55"/>
-      <c r="L34" s="54"/>
+      <c r="C34" s="57"/>
+      <c r="D34" s="58"/>
+      <c r="E34" s="57"/>
+      <c r="F34" s="58"/>
+      <c r="G34" s="57"/>
+      <c r="H34" s="59"/>
+      <c r="I34" s="58"/>
+      <c r="J34" s="57"/>
+      <c r="K34" s="59"/>
+      <c r="L34" s="58"/>
     </row>
     <row r="35" spans="2:12" ht="15.75" customHeight="1" thickBot="1">
       <c r="B35" s="49"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="54"/>
-      <c r="G35" s="53"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="54"/>
-      <c r="J35" s="53"/>
-      <c r="K35" s="55"/>
-      <c r="L35" s="54"/>
+      <c r="C35" s="57"/>
+      <c r="D35" s="58"/>
+      <c r="E35" s="57"/>
+      <c r="F35" s="58"/>
+      <c r="G35" s="57"/>
+      <c r="H35" s="59"/>
+      <c r="I35" s="58"/>
+      <c r="J35" s="57"/>
+      <c r="K35" s="59"/>
+      <c r="L35" s="58"/>
     </row>
     <row r="36" spans="2:12" ht="15.75" customHeight="1" thickBot="1">
       <c r="B36" s="49"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="54"/>
-      <c r="E36" s="53"/>
-      <c r="F36" s="54"/>
-      <c r="G36" s="53"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="54"/>
-      <c r="J36" s="53"/>
-      <c r="K36" s="55"/>
-      <c r="L36" s="54"/>
+      <c r="C36" s="57"/>
+      <c r="D36" s="58"/>
+      <c r="E36" s="57"/>
+      <c r="F36" s="58"/>
+      <c r="G36" s="57"/>
+      <c r="H36" s="59"/>
+      <c r="I36" s="58"/>
+      <c r="J36" s="57"/>
+      <c r="K36" s="59"/>
+      <c r="L36" s="58"/>
     </row>
     <row r="46" spans="2:12">
-      <c r="B46" s="89"/>
-      <c r="C46" s="52"/>
-      <c r="D46" s="52"/>
-      <c r="E46" s="52"/>
-      <c r="F46" s="52"/>
-      <c r="G46" s="90"/>
-      <c r="H46" s="90"/>
-      <c r="I46" s="90"/>
-      <c r="J46" s="90"/>
-      <c r="K46" s="90"/>
-      <c r="L46" s="90"/>
+      <c r="B46" s="52"/>
+      <c r="C46" s="93"/>
+      <c r="D46" s="93"/>
+      <c r="E46" s="93"/>
+      <c r="F46" s="93"/>
+      <c r="G46" s="94"/>
+      <c r="H46" s="94"/>
+      <c r="I46" s="94"/>
+      <c r="J46" s="94"/>
+      <c r="K46" s="94"/>
+      <c r="L46" s="94"/>
     </row>
     <row r="47" spans="2:12">
-      <c r="B47" s="89"/>
-      <c r="C47" s="52"/>
-      <c r="D47" s="52"/>
-      <c r="E47" s="52"/>
-      <c r="F47" s="52"/>
-      <c r="G47" s="52"/>
-      <c r="H47" s="52"/>
-      <c r="I47" s="52"/>
-      <c r="J47" s="52"/>
-      <c r="K47" s="52"/>
-      <c r="L47" s="52"/>
+      <c r="B47" s="52"/>
+      <c r="C47" s="93"/>
+      <c r="D47" s="93"/>
+      <c r="E47" s="93"/>
+      <c r="F47" s="93"/>
+      <c r="G47" s="93"/>
+      <c r="H47" s="93"/>
+      <c r="I47" s="93"/>
+      <c r="J47" s="93"/>
+      <c r="K47" s="93"/>
+      <c r="L47" s="93"/>
     </row>
     <row r="48" spans="2:12">
-      <c r="B48" s="89"/>
-      <c r="C48" s="52"/>
-      <c r="D48" s="52"/>
-      <c r="E48" s="52"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="52"/>
-      <c r="H48" s="52"/>
-      <c r="I48" s="52"/>
-      <c r="J48" s="52"/>
-      <c r="K48" s="52"/>
-      <c r="L48" s="52"/>
+      <c r="B48" s="52"/>
+      <c r="C48" s="93"/>
+      <c r="D48" s="93"/>
+      <c r="E48" s="93"/>
+      <c r="F48" s="93"/>
+      <c r="G48" s="93"/>
+      <c r="H48" s="93"/>
+      <c r="I48" s="93"/>
+      <c r="J48" s="93"/>
+      <c r="K48" s="93"/>
+      <c r="L48" s="93"/>
     </row>
     <row r="49" spans="2:12">
-      <c r="B49" s="89"/>
-      <c r="C49" s="52"/>
-      <c r="D49" s="52"/>
-      <c r="E49" s="52"/>
-      <c r="F49" s="52"/>
-      <c r="G49" s="52"/>
-      <c r="H49" s="52"/>
-      <c r="I49" s="52"/>
-      <c r="J49" s="52"/>
-      <c r="K49" s="52"/>
-      <c r="L49" s="52"/>
+      <c r="B49" s="52"/>
+      <c r="C49" s="93"/>
+      <c r="D49" s="93"/>
+      <c r="E49" s="93"/>
+      <c r="F49" s="93"/>
+      <c r="G49" s="93"/>
+      <c r="H49" s="93"/>
+      <c r="I49" s="93"/>
+      <c r="J49" s="93"/>
+      <c r="K49" s="93"/>
+      <c r="L49" s="93"/>
     </row>
     <row r="50" spans="2:12">
-      <c r="B50" s="89"/>
-      <c r="C50" s="52"/>
-      <c r="D50" s="52"/>
-      <c r="E50" s="52"/>
-      <c r="F50" s="52"/>
-      <c r="G50" s="90"/>
-      <c r="H50" s="90"/>
-      <c r="I50" s="90"/>
-      <c r="J50" s="90"/>
-      <c r="K50" s="90"/>
-      <c r="L50" s="90"/>
+      <c r="B50" s="52"/>
+      <c r="C50" s="93"/>
+      <c r="D50" s="93"/>
+      <c r="E50" s="93"/>
+      <c r="F50" s="93"/>
+      <c r="G50" s="94"/>
+      <c r="H50" s="94"/>
+      <c r="I50" s="94"/>
+      <c r="J50" s="94"/>
+      <c r="K50" s="94"/>
+      <c r="L50" s="94"/>
     </row>
     <row r="51" spans="2:12">
-      <c r="B51" s="89"/>
-      <c r="C51" s="52"/>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="52"/>
-      <c r="G51" s="52"/>
-      <c r="H51" s="52"/>
-      <c r="I51" s="52"/>
-      <c r="J51" s="52"/>
-      <c r="K51" s="52"/>
-      <c r="L51" s="52"/>
+      <c r="B51" s="52"/>
+      <c r="C51" s="93"/>
+      <c r="D51" s="93"/>
+      <c r="E51" s="93"/>
+      <c r="F51" s="93"/>
+      <c r="G51" s="93"/>
+      <c r="H51" s="93"/>
+      <c r="I51" s="93"/>
+      <c r="J51" s="93"/>
+      <c r="K51" s="93"/>
+      <c r="L51" s="93"/>
     </row>
     <row r="52" spans="2:12">
-      <c r="B52" s="89"/>
-      <c r="C52" s="52"/>
-      <c r="D52" s="52"/>
-      <c r="E52" s="52"/>
-      <c r="F52" s="52"/>
-      <c r="G52" s="52"/>
-      <c r="H52" s="52"/>
-      <c r="I52" s="52"/>
-      <c r="J52" s="52"/>
-      <c r="K52" s="52"/>
-      <c r="L52" s="52"/>
+      <c r="B52" s="52"/>
+      <c r="C52" s="93"/>
+      <c r="D52" s="93"/>
+      <c r="E52" s="93"/>
+      <c r="F52" s="93"/>
+      <c r="G52" s="93"/>
+      <c r="H52" s="93"/>
+      <c r="I52" s="93"/>
+      <c r="J52" s="93"/>
+      <c r="K52" s="93"/>
+      <c r="L52" s="93"/>
     </row>
     <row r="53" spans="2:12">
-      <c r="B53" s="89"/>
-      <c r="C53" s="52"/>
-      <c r="D53" s="52"/>
-      <c r="E53" s="52"/>
-      <c r="F53" s="52"/>
-      <c r="G53" s="52"/>
-      <c r="H53" s="52"/>
-      <c r="I53" s="52"/>
-      <c r="J53" s="52"/>
-      <c r="K53" s="52"/>
-      <c r="L53" s="52"/>
+      <c r="B53" s="52"/>
+      <c r="C53" s="93"/>
+      <c r="D53" s="93"/>
+      <c r="E53" s="93"/>
+      <c r="F53" s="93"/>
+      <c r="G53" s="93"/>
+      <c r="H53" s="93"/>
+      <c r="I53" s="93"/>
+      <c r="J53" s="93"/>
+      <c r="K53" s="93"/>
+      <c r="L53" s="93"/>
     </row>
     <row r="54" spans="2:12">
-      <c r="B54" s="89"/>
-      <c r="C54" s="52"/>
-      <c r="D54" s="52"/>
-      <c r="E54" s="52"/>
-      <c r="F54" s="52"/>
-      <c r="G54" s="52"/>
-      <c r="H54" s="52"/>
-      <c r="I54" s="52"/>
-      <c r="J54" s="52"/>
-      <c r="K54" s="52"/>
-      <c r="L54" s="52"/>
+      <c r="B54" s="52"/>
+      <c r="C54" s="93"/>
+      <c r="D54" s="93"/>
+      <c r="E54" s="93"/>
+      <c r="F54" s="93"/>
+      <c r="G54" s="93"/>
+      <c r="H54" s="93"/>
+      <c r="I54" s="93"/>
+      <c r="J54" s="93"/>
+      <c r="K54" s="93"/>
+      <c r="L54" s="93"/>
     </row>
     <row r="55" spans="2:12">
-      <c r="B55" s="89"/>
-      <c r="C55" s="52"/>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="52"/>
-      <c r="H55" s="52"/>
-      <c r="I55" s="52"/>
-      <c r="J55" s="52"/>
-      <c r="K55" s="52"/>
-      <c r="L55" s="52"/>
+      <c r="B55" s="52"/>
+      <c r="C55" s="93"/>
+      <c r="D55" s="93"/>
+      <c r="E55" s="93"/>
+      <c r="F55" s="93"/>
+      <c r="G55" s="93"/>
+      <c r="H55" s="93"/>
+      <c r="I55" s="93"/>
+      <c r="J55" s="93"/>
+      <c r="K55" s="93"/>
+      <c r="L55" s="93"/>
     </row>
   </sheetData>
   <mergeCells count="131">
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="G46:I46"/>
-    <mergeCell ref="J46:L46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="J47:L47"/>
     <mergeCell ref="C55:D55"/>
     <mergeCell ref="E55:F55"/>
     <mergeCell ref="G55:I55"/>
@@ -2516,10 +2514,6 @@
     <mergeCell ref="E54:F54"/>
     <mergeCell ref="G54:I54"/>
     <mergeCell ref="J54:L54"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="G51:I51"/>
-    <mergeCell ref="J51:L51"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="E52:F52"/>
     <mergeCell ref="G52:I52"/>
@@ -2532,6 +2526,10 @@
     <mergeCell ref="E50:F50"/>
     <mergeCell ref="G50:I50"/>
     <mergeCell ref="J50:L50"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="J51:L51"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="E48:F48"/>
     <mergeCell ref="G48:I48"/>
@@ -2544,7 +2542,14 @@
     <mergeCell ref="E36:F36"/>
     <mergeCell ref="G36:I36"/>
     <mergeCell ref="J36:L36"/>
-    <mergeCell ref="J33:L33"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="J46:L46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="J47:L47"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="G34:I34"/>
@@ -2612,6 +2617,9 @@
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="I6:J6"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="G33:I33"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="G30:I30"/>
@@ -2624,9 +2632,7 @@
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="G32:I32"/>
     <mergeCell ref="J32:L32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="J33:L33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2742,16 +2748,16 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="72" customHeight="1">
-      <c r="A11" s="2">
+      <c r="A11" s="55">
         <v>1</v>
       </c>
-      <c r="B11" s="91" t="s">
+      <c r="B11" s="53" t="s">
         <v>50</v>
       </c>
       <c r="C11" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="D11" s="91" t="s">
+      <c r="D11" s="53" t="s">
         <v>51</v>
       </c>
       <c r="E11" s="2"/>
@@ -2762,27 +2768,27 @@
         <v>52</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="I11" s="91" t="s">
+      <c r="I11" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J11" s="91" t="s">
+      <c r="J11" s="53" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="60">
-      <c r="A12" s="2">
+      <c r="A12" s="55">
         <v>2</v>
       </c>
-      <c r="B12" s="91" t="s">
+      <c r="B12" s="53" t="s">
         <v>54</v>
       </c>
       <c r="C12" s="51" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="91" t="s">
+      <c r="D12" s="53" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="91" t="s">
+      <c r="E12" s="53" t="s">
         <v>56</v>
       </c>
       <c r="F12" s="51" t="s">
@@ -2792,24 +2798,24 @@
         <v>58</v>
       </c>
       <c r="H12" s="2"/>
-      <c r="I12" s="91" t="s">
+      <c r="I12" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J12" s="91" t="s">
+      <c r="J12" s="53" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="105">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="91" t="s">
+      <c r="B13" s="53" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="91" t="s">
+      <c r="C13" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="D13" s="91" t="s">
+      <c r="D13" s="53" t="s">
         <v>62</v>
       </c>
       <c r="E13" s="50" t="s">
@@ -2824,21 +2830,21 @@
       <c r="H13" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="I13" s="91" t="s">
+      <c r="I13" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J13" s="91" t="s">
+      <c r="J13" s="53" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="75">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="55" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="91" t="s">
+      <c r="B14" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="91" t="s">
+      <c r="C14" s="53" t="s">
         <v>69</v>
       </c>
       <c r="D14" s="51" t="s">
@@ -2854,21 +2860,21 @@
         <v>68</v>
       </c>
       <c r="H14" s="2"/>
-      <c r="I14" s="91" t="s">
+      <c r="I14" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="J14" s="91" t="s">
+      <c r="J14" s="53" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="90">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="91" t="s">
+      <c r="B15" s="53" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="91" t="s">
+      <c r="C15" s="53" t="s">
         <v>74</v>
       </c>
       <c r="D15" s="51" t="s">
@@ -2884,21 +2890,21 @@
         <v>77</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="I15" s="91" t="s">
+      <c r="I15" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="J15" s="91" t="s">
+      <c r="J15" s="53" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="45">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="55" t="s">
         <v>80</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="56" t="s">
         <v>83</v>
       </c>
       <c r="D16" s="2"/>
@@ -2920,16 +2926,16 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="60">
-      <c r="A17" s="2">
+      <c r="A17" s="55">
         <v>3</v>
       </c>
-      <c r="B17" s="91" t="s">
+      <c r="B17" s="53" t="s">
         <v>88</v>
       </c>
       <c r="C17" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="D17" s="91" t="s">
+      <c r="D17" s="53" t="s">
         <v>89</v>
       </c>
       <c r="E17" s="2"/>
@@ -2948,196 +2954,196 @@
       </c>
     </row>
     <row r="18" spans="1:10" ht="30">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="55" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="91" t="s">
+      <c r="B18" s="53" t="s">
         <v>109</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="91" t="s">
+      <c r="D18" s="53" t="s">
         <v>89</v>
       </c>
       <c r="E18" s="2"/>
-      <c r="F18" s="91" t="s">
+      <c r="F18" s="53" t="s">
         <v>97</v>
       </c>
-      <c r="G18" s="91" t="s">
+      <c r="G18" s="53" t="s">
         <v>98</v>
       </c>
       <c r="H18" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="I18" s="91" t="s">
+      <c r="I18" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J18" s="91" t="s">
+      <c r="J18" s="53" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="45">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="55" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="91" t="s">
+      <c r="B19" s="53" t="s">
         <v>109</v>
       </c>
       <c r="C19" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="91" t="s">
+      <c r="D19" s="53" t="s">
         <v>89</v>
       </c>
       <c r="E19" s="2"/>
-      <c r="F19" s="91" t="s">
+      <c r="F19" s="53" t="s">
         <v>100</v>
       </c>
-      <c r="G19" s="91" t="s">
+      <c r="G19" s="53" t="s">
         <v>101</v>
       </c>
       <c r="H19" s="51" t="s">
         <v>102</v>
       </c>
-      <c r="I19" s="91" t="s">
+      <c r="I19" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J19" s="91" t="s">
+      <c r="J19" s="53" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="45">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="55" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="91" t="s">
+      <c r="B20" s="53" t="s">
         <v>109</v>
       </c>
       <c r="C20" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D20" s="91" t="s">
+      <c r="D20" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="E20" s="91"/>
-      <c r="F20" s="91" t="s">
+      <c r="E20" s="53"/>
+      <c r="F20" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="G20" s="91" t="s">
+      <c r="G20" s="53" t="s">
         <v>101</v>
       </c>
       <c r="H20" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="I20" s="91" t="s">
+      <c r="I20" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J20" s="91" t="s">
+      <c r="J20" s="53" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="45">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="55" t="s">
         <v>106</v>
       </c>
-      <c r="B21" s="91" t="s">
+      <c r="B21" s="53" t="s">
         <v>109</v>
       </c>
       <c r="C21" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="91" t="s">
+      <c r="D21" s="53" t="s">
         <v>107</v>
       </c>
-      <c r="E21" s="91"/>
-      <c r="F21" s="91" t="s">
+      <c r="E21" s="53"/>
+      <c r="F21" s="53" t="s">
         <v>108</v>
       </c>
-      <c r="G21" s="91" t="s">
+      <c r="G21" s="53" t="s">
         <v>101</v>
       </c>
       <c r="H21" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="I21" s="91" t="s">
+      <c r="I21" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="J21" s="91" t="s">
+      <c r="J21" s="53" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="45">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="55" t="s">
         <v>110</v>
       </c>
-      <c r="B22" s="91" t="s">
+      <c r="B22" s="53" t="s">
         <v>109</v>
       </c>
       <c r="C22" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D22" s="91" t="s">
+      <c r="D22" s="53" t="s">
         <v>111</v>
       </c>
-      <c r="E22" s="91"/>
-      <c r="F22" s="91" t="s">
+      <c r="E22" s="53"/>
+      <c r="F22" s="53" t="s">
         <v>100</v>
       </c>
-      <c r="G22" s="91" t="s">
+      <c r="G22" s="53" t="s">
         <v>101</v>
       </c>
       <c r="H22" s="51" t="s">
         <v>102</v>
       </c>
-      <c r="I22" s="91" t="s">
+      <c r="I22" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J22" s="91" t="s">
+      <c r="J22" s="53" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="45">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="55" t="s">
         <v>112</v>
       </c>
-      <c r="B23" s="91" t="s">
+      <c r="B23" s="53" t="s">
         <v>109</v>
       </c>
       <c r="C23" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D23" s="91" t="s">
+      <c r="D23" s="53" t="s">
         <v>111</v>
       </c>
-      <c r="E23" s="91"/>
-      <c r="F23" s="91" t="s">
+      <c r="E23" s="53"/>
+      <c r="F23" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="G23" s="91" t="s">
+      <c r="G23" s="53" t="s">
         <v>101</v>
       </c>
       <c r="H23" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="I23" s="91" t="s">
+      <c r="I23" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="J23" s="91" t="s">
+      <c r="J23" s="53" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:10">
-      <c r="A24" s="92"/>
-      <c r="B24" s="92"/>
-      <c r="C24" s="92"/>
-      <c r="D24" s="92"/>
-      <c r="E24" s="92"/>
-      <c r="F24" s="92"/>
-      <c r="G24" s="92"/>
-      <c r="H24" s="92"/>
-      <c r="I24" s="92"/>
-      <c r="J24" s="92"/>
+      <c r="A24" s="54"/>
+      <c r="B24" s="54"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="54"/>
+      <c r="G24" s="54"/>
+      <c r="H24" s="54"/>
+      <c r="I24" s="54"/>
+      <c r="J24" s="54"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="1"/>

</xml_diff>